<commit_message>
add the proj code to repo
</commit_message>
<xml_diff>
--- a/Resource/TestData.xlsx
+++ b/Resource/TestData.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\532252\IdeaProjects\sample1\Resource\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83944EA9-2830-43AA-B266-D98925D4606D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59E52A71-C803-43CB-8E05-A546C494F6F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="12">
   <si>
     <t>PASS</t>
   </si>
@@ -62,7 +62,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -77,7 +76,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -91,16 +90,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor indexed="10"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="none">
-        <fgColor indexed="42"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="none">
         <fgColor indexed="10"/>
       </patternFill>
     </fill>
@@ -132,15 +121,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -467,122 +454,122 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" s="0">
+      <c r="A2">
         <v>10</v>
       </c>
-      <c r="B2" s="0">
+      <c r="B2">
         <v>5</v>
       </c>
-      <c r="C2" t="s" s="0">
+      <c r="C2" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="0">
+      <c r="D2">
         <v>15</v>
       </c>
-      <c r="E2" t="n" s="0">
-        <v>15.0</v>
-      </c>
-      <c r="F2" t="s" s="4">
+      <c r="E2">
+        <v>15</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" s="0">
+      <c r="A3">
         <v>20</v>
       </c>
-      <c r="B3" s="0">
+      <c r="B3">
         <v>4</v>
       </c>
-      <c r="C3" t="s" s="0">
+      <c r="C3" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="0">
+      <c r="D3">
         <v>16</v>
       </c>
-      <c r="E3" t="n" s="0">
-        <v>16.0</v>
-      </c>
-      <c r="F3" t="s" s="4">
+      <c r="E3">
+        <v>16</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" s="0">
+      <c r="A4">
         <v>15</v>
       </c>
-      <c r="B4" s="0">
+      <c r="B4">
         <v>3</v>
       </c>
-      <c r="C4" t="s" s="0">
+      <c r="C4" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="0">
+      <c r="D4">
         <v>45</v>
       </c>
-      <c r="E4" t="n" s="0">
-        <v>45.0</v>
-      </c>
-      <c r="F4" t="s" s="4">
+      <c r="E4">
+        <v>45</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" s="0">
+      <c r="A5">
         <v>8</v>
       </c>
-      <c r="B5" s="0">
+      <c r="B5">
         <v>2</v>
       </c>
-      <c r="C5" t="s" s="0">
+      <c r="C5" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="0">
+      <c r="D5">
         <v>4</v>
       </c>
-      <c r="E5" t="n" s="0">
-        <v>4.0</v>
-      </c>
-      <c r="F5" t="s" s="4">
+      <c r="E5">
+        <v>4</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>3</v>
+      </c>
+      <c r="C6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6">
+        <v>12</v>
+      </c>
+      <c r="E6">
+        <v>12</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6" s="0">
-        <v>9</v>
-      </c>
-      <c r="B6" s="0">
-        <v>3</v>
-      </c>
-      <c r="C6" t="s" s="0">
-        <v>7</v>
-      </c>
-      <c r="D6" s="0">
-        <v>12</v>
-      </c>
-      <c r="E6" t="n" s="0">
-        <v>12.0</v>
-      </c>
-      <c r="F6" t="s" s="4">
-        <v>0</v>
-      </c>
-    </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A7" s="0">
+      <c r="A7">
         <v>100</v>
       </c>
-      <c r="B7" s="0">
+      <c r="B7">
         <v>25</v>
       </c>
-      <c r="C7" t="s" s="0">
+      <c r="C7" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="0">
+      <c r="D7">
         <v>4</v>
       </c>
-      <c r="E7" t="n" s="0">
-        <v>4.0</v>
-      </c>
-      <c r="F7" t="s" s="4">
+      <c r="E7">
+        <v>4</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>0</v>
       </c>
     </row>

</xml_diff>